<commit_message>
Load dotenv credentials in Nattome pipeline CLIs
</commit_message>
<xml_diff>
--- a/outputs/reports/2026-05-06/20260506T134530Z_debug/top5_angle_planning_sheet_2026-05-06.xlsx
+++ b/outputs/reports/2026-05-06/20260506T134530Z_debug/top5_angle_planning_sheet_2026-05-06.xlsx
@@ -288,7 +288,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>telegram-video</t>
+          <t>missing-gemini</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -298,34 +298,34 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@creator/video/telegram</t>
+          <t>https://www.tiktok.com/@creator/video/twolayer</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Acid reflux stomach tip</t>
+          <t>Bloating after meals gut health routine</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>90000</v>
+        <v>120000</v>
       </c>
       <c r="G2" t="n">
-        <v>9000</v>
+        <v>12000</v>
       </c>
       <c r="H2" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="I2" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1722</v>
+        <v>0.1833</v>
       </c>
       <c r="K2" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4801</v>
+        <v>1.2969</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -334,7 +334,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Gemini API key is missing; set GEMINI_API_KEY; missing Gemini visual evidence; missing Gemini visible text evidence</t>
+          <t>Gemini API key is missing; set GEMINI_API_KEY; Gemini visible text evidence missing despite expected text; missing Gemini visual evidence</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -359,7 +359,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>DR for faster relief moments around reflux, heartburn, or gastric discomfort.</t>
+          <t>DH for daily digestive maintenance and routine support.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">

</xml_diff>